<commit_message>
Configure permanent Vercel domain brush-iq.vercel.app & update Selenium test target
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:34 am</t>
+    <t>28/7/2026, 5:47:12 pm</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>35.73 seconds</t>
+    <t>38.09 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,109 +3949,109 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:02 am</t>
-  </si>
-  <si>
-    <t>2.05s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:05 am</t>
-  </si>
-  <si>
-    <t>2.80s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:07 am</t>
+    <t>28/7/2026, 5:46:39 pm</t>
   </si>
   <si>
     <t>2.48s</t>
   </si>
   <si>
+    <t>28/7/2026, 5:46:42 pm</t>
+  </si>
+  <si>
+    <t>2.49s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:44 pm</t>
+  </si>
+  <si>
+    <t>2.42s</t>
+  </si>
+  <si>
     <t>0.15s</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:10 am</t>
-  </si>
-  <si>
-    <t>2.59s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:12 am</t>
-  </si>
-  <si>
-    <t>2.33s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:14 am</t>
-  </si>
-  <si>
-    <t>2.24s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:16 am</t>
-  </si>
-  <si>
-    <t>2.34s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:19 am</t>
-  </si>
-  <si>
-    <t>2.11s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:21 am</t>
-  </si>
-  <si>
-    <t>1.96s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:24 am</t>
-  </si>
-  <si>
-    <t>2.84s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:26 am</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:28 am</t>
-  </si>
-  <si>
-    <t>2.02s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:30 am</t>
-  </si>
-  <si>
-    <t>2.28s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:31 am</t>
-  </si>
-  <si>
-    <t>0.30s</t>
-  </si>
-  <si>
-    <t>0.29s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:32 am</t>
-  </si>
-  <si>
-    <t>0.31s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:33 am</t>
-  </si>
-  <si>
-    <t>0.37s</t>
-  </si>
-  <si>
-    <t>0.28s</t>
-  </si>
-  <si>
-    <t>0.19s</t>
+    <t>28/7/2026, 5:46:47 pm</t>
+  </si>
+  <si>
+    <t>2.64s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:49 pm</t>
+  </si>
+  <si>
+    <t>2.31s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:52 pm</t>
+  </si>
+  <si>
+    <t>2.90s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:54 pm</t>
+  </si>
+  <si>
+    <t>2.21s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:56 pm</t>
+  </si>
+  <si>
+    <t>2.13s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:46:58 pm</t>
+  </si>
+  <si>
+    <t>2.03s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:01 pm</t>
+  </si>
+  <si>
+    <t>2.52s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:03 pm</t>
+  </si>
+  <si>
+    <t>2.25s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:05 pm</t>
+  </si>
+  <si>
+    <t>2.07s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:08 pm</t>
+  </si>
+  <si>
+    <t>0.36s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:09 pm</t>
+  </si>
+  <si>
+    <t>0.35s</t>
+  </si>
+  <si>
+    <t>0.42s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:10 pm</t>
+  </si>
+  <si>
+    <t>0.40s</t>
+  </si>
+  <si>
+    <t>0.34s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 5:47:11 pm</t>
+  </si>
+  <si>
+    <t>0.27s</t>
   </si>
 </sst>
 </file>
@@ -15180,7 +15180,7 @@
         <v>9</v>
       </c>
       <c r="C41" t="s">
-        <v>1323</v>
+        <v>1333</v>
       </c>
       <c r="D41" t="s">
         <v>35</v>
@@ -15188,13 +15188,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
       </c>
       <c r="C42" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="D42" t="s">
         <v>35</v>
@@ -15202,7 +15202,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -15216,7 +15216,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -15230,7 +15230,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -15244,7 +15244,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -15258,7 +15258,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -15272,7 +15272,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -15286,7 +15286,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -15300,7 +15300,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -15314,7 +15314,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -15328,7 +15328,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -15342,7 +15342,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -15356,7 +15356,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -15370,7 +15370,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -15384,7 +15384,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -15398,7 +15398,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B57" t="s">
         <v>9</v>
@@ -15412,7 +15412,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -15426,7 +15426,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
@@ -15440,7 +15440,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
@@ -15454,7 +15454,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B61" t="s">
         <v>9</v>
@@ -15468,13 +15468,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B62" t="s">
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>1336</v>
+        <v>1325</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15482,7 +15482,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -15496,7 +15496,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
@@ -15510,7 +15510,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -15524,7 +15524,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B66" t="s">
         <v>9</v>
@@ -15538,7 +15538,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -15552,7 +15552,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -15566,7 +15566,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -15580,7 +15580,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
@@ -15594,7 +15594,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B71" t="s">
         <v>9</v>
@@ -15608,7 +15608,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B72" t="s">
         <v>9</v>
@@ -15622,7 +15622,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
@@ -15636,7 +15636,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B74" t="s">
         <v>9</v>
@@ -15650,7 +15650,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B75" t="s">
         <v>9</v>
@@ -15664,7 +15664,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -15678,7 +15678,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
@@ -15692,7 +15692,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
@@ -15706,7 +15706,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
@@ -15720,7 +15720,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -15734,7 +15734,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
@@ -15748,13 +15748,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
         <v>1337</v>
-      </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
-      <c r="C82" t="s">
-        <v>1338</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -15762,7 +15762,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
@@ -15776,7 +15776,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -15790,7 +15790,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -15804,7 +15804,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -15818,7 +15818,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B87" t="s">
         <v>9</v>
@@ -15832,7 +15832,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B88" t="s">
         <v>9</v>
@@ -15846,7 +15846,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -15860,7 +15860,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -15874,7 +15874,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -15888,7 +15888,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -15902,7 +15902,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B93" t="s">
         <v>9</v>
@@ -15916,7 +15916,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B94" t="s">
         <v>9</v>
@@ -15930,7 +15930,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B95" t="s">
         <v>9</v>
@@ -15944,7 +15944,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B96" t="s">
         <v>9</v>
@@ -15958,7 +15958,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -15972,7 +15972,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B98" t="s">
         <v>9</v>
@@ -15986,7 +15986,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -16000,7 +16000,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B100" t="s">
         <v>9</v>
@@ -16014,7 +16014,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -16028,7 +16028,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B102" t="s">
         <v>9</v>
@@ -16042,7 +16042,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B103" t="s">
         <v>9</v>
@@ -16056,7 +16056,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B104" t="s">
         <v>9</v>
@@ -16070,7 +16070,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -16084,7 +16084,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B106" t="s">
         <v>9</v>
@@ -16098,7 +16098,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
@@ -16112,7 +16112,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B108" t="s">
         <v>9</v>
@@ -16126,7 +16126,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B109" t="s">
         <v>9</v>
@@ -16140,7 +16140,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B110" t="s">
         <v>9</v>
@@ -16154,7 +16154,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -16168,13 +16168,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B112" t="s">
         <v>9</v>
       </c>
       <c r="C112" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="D112" t="s">
         <v>35</v>
@@ -16182,7 +16182,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B113" t="s">
         <v>9</v>
@@ -16196,7 +16196,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B114" t="s">
         <v>9</v>
@@ -16210,7 +16210,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B115" t="s">
         <v>9</v>
@@ -16224,7 +16224,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B116" t="s">
         <v>9</v>
@@ -16238,7 +16238,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B117" t="s">
         <v>9</v>
@@ -16252,7 +16252,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B118" t="s">
         <v>9</v>
@@ -16266,7 +16266,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B119" t="s">
         <v>9</v>
@@ -16280,7 +16280,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B120" t="s">
         <v>9</v>
@@ -16294,7 +16294,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B121" t="s">
         <v>9</v>
@@ -16308,7 +16308,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B122" t="s">
         <v>9</v>
@@ -16322,7 +16322,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B123" t="s">
         <v>9</v>
@@ -16336,7 +16336,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B124" t="s">
         <v>9</v>
@@ -16350,7 +16350,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B125" t="s">
         <v>9</v>
@@ -16364,7 +16364,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B126" t="s">
         <v>9</v>
@@ -16378,7 +16378,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -16392,7 +16392,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -16406,7 +16406,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -16420,7 +16420,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -16434,7 +16434,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -16448,7 +16448,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -16462,7 +16462,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -16476,7 +16476,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -16490,7 +16490,7 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
@@ -16504,7 +16504,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -16518,13 +16518,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B137" t="s">
         <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="D137" t="s">
         <v>35</v>
@@ -16532,7 +16532,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -16546,7 +16546,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -16560,7 +16560,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -16574,7 +16574,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -16588,7 +16588,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -16602,7 +16602,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -16616,7 +16616,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -16630,7 +16630,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -16644,7 +16644,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -16658,7 +16658,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -16672,7 +16672,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -16686,7 +16686,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -16700,7 +16700,7 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -16714,7 +16714,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -16728,7 +16728,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -16742,7 +16742,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -16756,7 +16756,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -16770,7 +16770,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -16784,7 +16784,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -16798,7 +16798,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -16812,7 +16812,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -16826,7 +16826,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -16840,7 +16840,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -16854,7 +16854,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -16868,7 +16868,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -16882,7 +16882,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -16896,7 +16896,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -16910,7 +16910,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -16924,7 +16924,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -16938,13 +16938,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
       </c>
       <c r="C167" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="D167" t="s">
         <v>35</v>
@@ -16952,7 +16952,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -16966,7 +16966,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -16980,7 +16980,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -16994,7 +16994,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -17008,7 +17008,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -17022,7 +17022,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -17036,7 +17036,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -17050,7 +17050,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B175" t="s">
         <v>9</v>
@@ -17064,7 +17064,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -17078,7 +17078,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -17092,7 +17092,7 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -17106,7 +17106,7 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -17120,7 +17120,7 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -17134,7 +17134,7 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -17148,7 +17148,7 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -17162,7 +17162,7 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -17176,7 +17176,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -17190,7 +17190,7 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -17204,7 +17204,7 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -17218,7 +17218,7 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -17232,7 +17232,7 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -17246,7 +17246,7 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -17260,7 +17260,7 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -17274,7 +17274,7 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -17288,13 +17288,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
       </c>
       <c r="C192" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17302,7 +17302,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17316,7 +17316,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17330,7 +17330,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17344,7 +17344,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17358,7 +17358,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17372,7 +17372,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17386,7 +17386,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17400,7 +17400,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17414,7 +17414,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17428,7 +17428,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17442,7 +17442,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17456,7 +17456,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17470,7 +17470,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17484,7 +17484,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17498,7 +17498,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17512,7 +17512,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17526,7 +17526,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17540,7 +17540,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17554,7 +17554,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17568,7 +17568,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17582,7 +17582,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17596,7 +17596,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17610,7 +17610,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17624,7 +17624,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17638,7 +17638,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17652,7 +17652,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17666,7 +17666,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17680,7 +17680,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17694,7 +17694,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17708,13 +17708,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
       </c>
       <c r="C222" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="D222" t="s">
         <v>35</v>
@@ -17722,7 +17722,7 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -17736,7 +17736,7 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -17750,7 +17750,7 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -17764,7 +17764,7 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -17778,7 +17778,7 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -17792,7 +17792,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -17806,7 +17806,7 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -17820,7 +17820,7 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -17834,7 +17834,7 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -17848,7 +17848,7 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>
@@ -17862,7 +17862,7 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B233" t="s">
         <v>9</v>
@@ -17876,7 +17876,7 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B234" t="s">
         <v>9</v>
@@ -17890,7 +17890,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B235" t="s">
         <v>9</v>
@@ -17904,7 +17904,7 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B236" t="s">
         <v>9</v>
@@ -17918,7 +17918,7 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B237" t="s">
         <v>9</v>
@@ -17932,7 +17932,7 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B238" t="s">
         <v>9</v>
@@ -17946,7 +17946,7 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B239" t="s">
         <v>9</v>
@@ -17960,7 +17960,7 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B240" t="s">
         <v>9</v>
@@ -17974,7 +17974,7 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B241" t="s">
         <v>9</v>
@@ -17988,7 +17988,7 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B242" t="s">
         <v>9</v>
@@ -18002,7 +18002,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B243" t="s">
         <v>9</v>
@@ -18016,7 +18016,7 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B244" t="s">
         <v>9</v>
@@ -18030,7 +18030,7 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B245" t="s">
         <v>9</v>
@@ -18044,7 +18044,7 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B246" t="s">
         <v>9</v>
@@ -18058,13 +18058,13 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B247" t="s">
         <v>9</v>
       </c>
       <c r="C247" t="s">
-        <v>1343</v>
+        <v>1337</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18072,7 +18072,7 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B248" t="s">
         <v>9</v>
@@ -18086,7 +18086,7 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B249" t="s">
         <v>9</v>
@@ -18100,7 +18100,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B250" t="s">
         <v>9</v>
@@ -18114,7 +18114,7 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B251" t="s">
         <v>9</v>
@@ -18128,7 +18128,7 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B252" t="s">
         <v>9</v>
@@ -18142,7 +18142,7 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B253" t="s">
         <v>9</v>
@@ -18156,7 +18156,7 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B254" t="s">
         <v>9</v>
@@ -18170,7 +18170,7 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B255" t="s">
         <v>9</v>
@@ -18184,7 +18184,7 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B256" t="s">
         <v>9</v>
@@ -18198,7 +18198,7 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B257" t="s">
         <v>9</v>
@@ -18212,7 +18212,7 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B258" t="s">
         <v>9</v>
@@ -18226,7 +18226,7 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B259" t="s">
         <v>9</v>
@@ -18240,7 +18240,7 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B260" t="s">
         <v>9</v>
@@ -18254,7 +18254,7 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B261" t="s">
         <v>9</v>
@@ -18268,7 +18268,7 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B262" t="s">
         <v>9</v>
@@ -18282,7 +18282,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B263" t="s">
         <v>9</v>
@@ -18296,7 +18296,7 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B264" t="s">
         <v>9</v>
@@ -18310,7 +18310,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B265" t="s">
         <v>9</v>
@@ -18324,7 +18324,7 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B266" t="s">
         <v>9</v>
@@ -18338,7 +18338,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B267" t="s">
         <v>9</v>
@@ -18352,7 +18352,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B268" t="s">
         <v>9</v>
@@ -18366,7 +18366,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B269" t="s">
         <v>9</v>
@@ -18380,7 +18380,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B270" t="s">
         <v>9</v>
@@ -18394,7 +18394,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="B271" t="s">
         <v>9</v>
@@ -18408,13 +18408,13 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B272" t="s">
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1344</v>
+        <v>1339</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18422,7 +18422,7 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B273" t="s">
         <v>9</v>
@@ -18436,7 +18436,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B274" t="s">
         <v>9</v>
@@ -18450,7 +18450,7 @@
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B275" t="s">
         <v>9</v>
@@ -18464,7 +18464,7 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B276" t="s">
         <v>9</v>
@@ -18478,7 +18478,7 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B277" t="s">
         <v>9</v>
@@ -18492,7 +18492,7 @@
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B278" t="s">
         <v>9</v>
@@ -18506,7 +18506,7 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B279" t="s">
         <v>9</v>
@@ -18520,7 +18520,7 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B280" t="s">
         <v>9</v>
@@ -18534,7 +18534,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B281" t="s">
         <v>9</v>
@@ -18548,7 +18548,7 @@
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B282" t="s">
         <v>9</v>
@@ -18562,7 +18562,7 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B283" t="s">
         <v>9</v>
@@ -18576,7 +18576,7 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B284" t="s">
         <v>9</v>
@@ -18590,7 +18590,7 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B285" t="s">
         <v>9</v>
@@ -18604,7 +18604,7 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B286" t="s">
         <v>9</v>
@@ -18618,7 +18618,7 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B287" t="s">
         <v>9</v>
@@ -18632,7 +18632,7 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B288" t="s">
         <v>9</v>
@@ -18646,7 +18646,7 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B289" t="s">
         <v>9</v>
@@ -18660,7 +18660,7 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B290" t="s">
         <v>9</v>
@@ -18674,7 +18674,7 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B291" t="s">
         <v>9</v>
@@ -18688,7 +18688,7 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B292" t="s">
         <v>9</v>
@@ -18702,7 +18702,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B293" t="s">
         <v>9</v>
@@ -18716,7 +18716,7 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B294" t="s">
         <v>9</v>
@@ -18730,7 +18730,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B295" t="s">
         <v>9</v>
@@ -18744,7 +18744,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>1342</v>
+        <v>7</v>
       </c>
       <c r="B296" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Phase 6: Selenium E2E Framework Execution (310/310 test cases passed)
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1349">
   <si>
     <t>Metric</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 5:47:12 pm</t>
+    <t>28/7/2026, 6:21:19 pm</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>38.09 seconds</t>
+    <t>39.89 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,106 +3949,115 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 5:46:39 pm</t>
-  </si>
-  <si>
-    <t>2.48s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:42 pm</t>
-  </si>
-  <si>
-    <t>2.49s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:44 pm</t>
-  </si>
-  <si>
-    <t>2.42s</t>
+    <t>28/7/2026, 6:20:43 pm</t>
+  </si>
+  <si>
+    <t>2.03s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:20:46 pm</t>
+  </si>
+  <si>
+    <t>2.66s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:20:49 pm</t>
+  </si>
+  <si>
+    <t>2.58s</t>
   </si>
   <si>
     <t>0.15s</t>
   </si>
   <si>
-    <t>28/7/2026, 5:46:47 pm</t>
-  </si>
-  <si>
-    <t>2.64s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:49 pm</t>
-  </si>
-  <si>
-    <t>2.31s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:52 pm</t>
-  </si>
-  <si>
-    <t>2.90s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:54 pm</t>
+    <t>28/7/2026, 6:20:51 pm</t>
+  </si>
+  <si>
+    <t>2.47s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:20:54 pm</t>
+  </si>
+  <si>
+    <t>2.41s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:20:56 pm</t>
+  </si>
+  <si>
+    <t>2.79s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:20:59 pm</t>
+  </si>
+  <si>
+    <t>2.72s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:01 pm</t>
+  </si>
+  <si>
+    <t>2.08s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:03 pm</t>
+  </si>
+  <si>
+    <t>2.04s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:07 pm</t>
+  </si>
+  <si>
+    <t>3.31s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:09 pm</t>
+  </si>
+  <si>
+    <t>2.32s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:11 pm</t>
+  </si>
+  <si>
+    <t>2.13s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:14 pm</t>
   </si>
   <si>
     <t>2.21s</t>
   </si>
   <si>
-    <t>28/7/2026, 5:46:56 pm</t>
-  </si>
-  <si>
-    <t>2.13s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:46:58 pm</t>
-  </si>
-  <si>
-    <t>2.03s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:01 pm</t>
-  </si>
-  <si>
-    <t>2.52s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:03 pm</t>
-  </si>
-  <si>
-    <t>2.25s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:05 pm</t>
-  </si>
-  <si>
-    <t>2.07s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:08 pm</t>
-  </si>
-  <si>
-    <t>0.36s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:09 pm</t>
+    <t>0.40s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:15 pm</t>
+  </si>
+  <si>
+    <t>0.56s</t>
+  </si>
+  <si>
+    <t>0.00s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:16 pm</t>
   </si>
   <si>
     <t>0.35s</t>
   </si>
   <si>
-    <t>0.42s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:10 pm</t>
-  </si>
-  <si>
-    <t>0.40s</t>
-  </si>
-  <si>
-    <t>0.34s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 5:47:11 pm</t>
+    <t>28/7/2026, 6:21:17 pm</t>
+  </si>
+  <si>
+    <t>0.38s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:21:18 pm</t>
+  </si>
+  <si>
+    <t>0.41s</t>
   </si>
   <si>
     <t>0.27s</t>
@@ -15474,7 +15483,7 @@
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>1325</v>
+        <v>1337</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15754,7 +15763,7 @@
         <v>9</v>
       </c>
       <c r="C82" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -16168,13 +16177,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B112" t="s">
         <v>9</v>
       </c>
       <c r="C112" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="D112" t="s">
         <v>35</v>
@@ -16182,7 +16191,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B113" t="s">
         <v>9</v>
@@ -16196,7 +16205,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B114" t="s">
         <v>9</v>
@@ -16210,7 +16219,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B115" t="s">
         <v>9</v>
@@ -16224,7 +16233,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B116" t="s">
         <v>9</v>
@@ -16238,7 +16247,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B117" t="s">
         <v>9</v>
@@ -16252,7 +16261,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B118" t="s">
         <v>9</v>
@@ -16266,7 +16275,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B119" t="s">
         <v>9</v>
@@ -16280,7 +16289,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B120" t="s">
         <v>9</v>
@@ -16294,7 +16303,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B121" t="s">
         <v>9</v>
@@ -16308,7 +16317,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B122" t="s">
         <v>9</v>
@@ -16322,7 +16331,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B123" t="s">
         <v>9</v>
@@ -16336,7 +16345,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B124" t="s">
         <v>9</v>
@@ -16350,7 +16359,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B125" t="s">
         <v>9</v>
@@ -16364,7 +16373,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B126" t="s">
         <v>9</v>
@@ -16378,7 +16387,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -16392,7 +16401,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -16406,7 +16415,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -16420,7 +16429,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -16434,7 +16443,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -16448,7 +16457,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -16462,7 +16471,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -16476,7 +16485,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -16490,13 +16499,13 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
       </c>
       <c r="C135" t="s">
-        <v>1317</v>
+        <v>1341</v>
       </c>
       <c r="D135" t="s">
         <v>35</v>
@@ -16504,7 +16513,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -16518,13 +16527,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B137" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137" t="s">
         <v>1338</v>
-      </c>
-      <c r="B137" t="s">
-        <v>9</v>
-      </c>
-      <c r="C137" t="s">
-        <v>1340</v>
       </c>
       <c r="D137" t="s">
         <v>35</v>
@@ -16532,7 +16541,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -16546,7 +16555,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -16560,7 +16569,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -16574,7 +16583,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -16588,7 +16597,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -16602,7 +16611,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -16616,7 +16625,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -16630,7 +16639,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -16644,7 +16653,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -16658,7 +16667,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -16672,7 +16681,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -16686,7 +16695,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -16700,7 +16709,7 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -16714,7 +16723,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -16728,7 +16737,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -16742,7 +16751,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -16756,7 +16765,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -16770,7 +16779,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -16784,7 +16793,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -16798,7 +16807,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -16812,7 +16821,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -16826,7 +16835,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -16840,7 +16849,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -16854,7 +16863,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -16868,7 +16877,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -16882,7 +16891,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -16896,7 +16905,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -16910,7 +16919,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -16924,7 +16933,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -16938,13 +16947,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
       </c>
       <c r="C167" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="D167" t="s">
         <v>35</v>
@@ -16952,7 +16961,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -16966,7 +16975,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -16980,7 +16989,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -16994,7 +17003,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -17008,7 +17017,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -17022,7 +17031,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -17036,7 +17045,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -17050,7 +17059,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B175" t="s">
         <v>9</v>
@@ -17064,7 +17073,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -17078,7 +17087,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -17092,7 +17101,7 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -17106,7 +17115,7 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -17120,7 +17129,7 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -17134,7 +17143,7 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -17148,7 +17157,7 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -17162,7 +17171,7 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -17176,7 +17185,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -17190,7 +17199,7 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -17204,7 +17213,7 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -17218,7 +17227,7 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -17232,7 +17241,7 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -17246,7 +17255,7 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -17260,7 +17269,7 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -17274,7 +17283,7 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -17288,13 +17297,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
       </c>
       <c r="C192" t="s">
-        <v>1343</v>
+        <v>1345</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17302,7 +17311,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17316,7 +17325,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17330,7 +17339,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17344,7 +17353,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17358,7 +17367,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17372,7 +17381,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17386,7 +17395,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17400,7 +17409,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17414,7 +17423,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17428,7 +17437,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17442,7 +17451,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17456,7 +17465,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17470,7 +17479,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17484,7 +17493,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17498,7 +17507,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17512,7 +17521,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17526,7 +17535,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17540,7 +17549,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17554,7 +17563,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17568,7 +17577,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17582,7 +17591,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17596,7 +17605,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17610,7 +17619,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17624,7 +17633,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17638,7 +17647,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17652,7 +17661,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17666,7 +17675,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17680,7 +17689,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17694,7 +17703,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1341</v>
+        <v>1344</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17714,7 +17723,7 @@
         <v>9</v>
       </c>
       <c r="C222" t="s">
-        <v>1337</v>
+        <v>1345</v>
       </c>
       <c r="D222" t="s">
         <v>35</v>
@@ -17924,7 +17933,7 @@
         <v>9</v>
       </c>
       <c r="C237" t="s">
-        <v>1317</v>
+        <v>1341</v>
       </c>
       <c r="D237" t="s">
         <v>35</v>
@@ -18058,13 +18067,13 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B247" t="s">
         <v>9</v>
       </c>
       <c r="C247" t="s">
-        <v>1337</v>
+        <v>1345</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18072,7 +18081,7 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B248" t="s">
         <v>9</v>
@@ -18086,7 +18095,7 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B249" t="s">
         <v>9</v>
@@ -18100,7 +18109,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B250" t="s">
         <v>9</v>
@@ -18114,7 +18123,7 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B251" t="s">
         <v>9</v>
@@ -18128,7 +18137,7 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B252" t="s">
         <v>9</v>
@@ -18142,7 +18151,7 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B253" t="s">
         <v>9</v>
@@ -18156,7 +18165,7 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B254" t="s">
         <v>9</v>
@@ -18170,7 +18179,7 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B255" t="s">
         <v>9</v>
@@ -18184,7 +18193,7 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B256" t="s">
         <v>9</v>
@@ -18198,7 +18207,7 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B257" t="s">
         <v>9</v>
@@ -18212,7 +18221,7 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B258" t="s">
         <v>9</v>
@@ -18226,7 +18235,7 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B259" t="s">
         <v>9</v>
@@ -18240,7 +18249,7 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B260" t="s">
         <v>9</v>
@@ -18254,7 +18263,7 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B261" t="s">
         <v>9</v>
@@ -18268,7 +18277,7 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B262" t="s">
         <v>9</v>
@@ -18282,7 +18291,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B263" t="s">
         <v>9</v>
@@ -18296,7 +18305,7 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B264" t="s">
         <v>9</v>
@@ -18310,7 +18319,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B265" t="s">
         <v>9</v>
@@ -18324,7 +18333,7 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B266" t="s">
         <v>9</v>
@@ -18338,7 +18347,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B267" t="s">
         <v>9</v>
@@ -18352,7 +18361,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B268" t="s">
         <v>9</v>
@@ -18366,7 +18375,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B269" t="s">
         <v>9</v>
@@ -18380,7 +18389,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B270" t="s">
         <v>9</v>
@@ -18394,7 +18403,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="B271" t="s">
         <v>9</v>
@@ -18408,13 +18417,13 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B272" t="s">
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1339</v>
+        <v>1347</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18422,7 +18431,7 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B273" t="s">
         <v>9</v>
@@ -18436,7 +18445,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B274" t="s">
         <v>9</v>
@@ -18450,7 +18459,7 @@
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B275" t="s">
         <v>9</v>
@@ -18464,7 +18473,7 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B276" t="s">
         <v>9</v>
@@ -18478,7 +18487,7 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B277" t="s">
         <v>9</v>
@@ -18492,7 +18501,7 @@
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B278" t="s">
         <v>9</v>
@@ -18506,7 +18515,7 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B279" t="s">
         <v>9</v>
@@ -18520,7 +18529,7 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B280" t="s">
         <v>9</v>
@@ -18534,7 +18543,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B281" t="s">
         <v>9</v>
@@ -18548,7 +18557,7 @@
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B282" t="s">
         <v>9</v>
@@ -18562,7 +18571,7 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B283" t="s">
         <v>9</v>
@@ -18576,7 +18585,7 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B284" t="s">
         <v>9</v>
@@ -18590,7 +18599,7 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B285" t="s">
         <v>9</v>
@@ -18604,7 +18613,7 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B286" t="s">
         <v>9</v>
@@ -18618,7 +18627,7 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B287" t="s">
         <v>9</v>
@@ -18632,7 +18641,7 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B288" t="s">
         <v>9</v>
@@ -18646,7 +18655,7 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B289" t="s">
         <v>9</v>
@@ -18660,7 +18669,7 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B290" t="s">
         <v>9</v>
@@ -18674,7 +18683,7 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B291" t="s">
         <v>9</v>
@@ -18688,7 +18697,7 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B292" t="s">
         <v>9</v>
@@ -18702,7 +18711,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B293" t="s">
         <v>9</v>
@@ -18716,7 +18725,7 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B294" t="s">
         <v>9</v>
@@ -18730,7 +18739,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B295" t="s">
         <v>9</v>
@@ -18744,7 +18753,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>7</v>
+        <v>1346</v>
       </c>
       <c r="B296" t="s">
         <v>9</v>
@@ -18764,7 +18773,7 @@
         <v>9</v>
       </c>
       <c r="C297" t="s">
-        <v>1345</v>
+        <v>1348</v>
       </c>
       <c r="D297" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
Fix production registration: added auto-migration module on boot, enhanced auth logging, removed non-functional Google button
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1346">
   <si>
     <t>Metric</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 6:21:19 pm</t>
+    <t>28/7/2026, 6:32:41 pm</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>39.89 seconds</t>
+    <t>39.91 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,118 +3949,109 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 6:20:43 pm</t>
-  </si>
-  <si>
-    <t>2.03s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:20:46 pm</t>
-  </si>
-  <si>
-    <t>2.66s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:20:49 pm</t>
-  </si>
-  <si>
-    <t>2.58s</t>
+    <t>28/7/2026, 6:32:05 pm</t>
+  </si>
+  <si>
+    <t>2.06s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:07 pm</t>
+  </si>
+  <si>
+    <t>2.85s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:10 pm</t>
+  </si>
+  <si>
+    <t>2.43s</t>
   </si>
   <si>
     <t>0.15s</t>
   </si>
   <si>
-    <t>28/7/2026, 6:20:51 pm</t>
-  </si>
-  <si>
-    <t>2.47s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:20:54 pm</t>
-  </si>
-  <si>
-    <t>2.41s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:20:56 pm</t>
-  </si>
-  <si>
-    <t>2.79s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:20:59 pm</t>
-  </si>
-  <si>
-    <t>2.72s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:01 pm</t>
-  </si>
-  <si>
-    <t>2.08s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:03 pm</t>
-  </si>
-  <si>
-    <t>2.04s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:07 pm</t>
-  </si>
-  <si>
-    <t>3.31s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:09 pm</t>
-  </si>
-  <si>
-    <t>2.32s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:11 pm</t>
-  </si>
-  <si>
-    <t>2.13s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:14 pm</t>
+    <t>28/7/2026, 6:32:12 pm</t>
+  </si>
+  <si>
+    <t>2.48s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:15 pm</t>
+  </si>
+  <si>
+    <t>2.56s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:17 pm</t>
+  </si>
+  <si>
+    <t>2.51s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:20 pm</t>
+  </si>
+  <si>
+    <t>2.71s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:22 pm</t>
+  </si>
+  <si>
+    <t>2.18s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:25 pm</t>
+  </si>
+  <si>
+    <t>2.20s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:28 pm</t>
+  </si>
+  <si>
+    <t>2.93s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:31 pm</t>
+  </si>
+  <si>
+    <t>2.46s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:33 pm</t>
   </si>
   <si>
     <t>2.21s</t>
   </si>
   <si>
+    <t>28/7/2026, 6:32:36 pm</t>
+  </si>
+  <si>
+    <t>0.37s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:37 pm</t>
+  </si>
+  <si>
+    <t>0.38s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:38 pm</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:39 pm</t>
+  </si>
+  <si>
+    <t>0.36s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 6:32:40 pm</t>
+  </si>
+  <si>
     <t>0.40s</t>
   </si>
   <si>
-    <t>28/7/2026, 6:21:15 pm</t>
-  </si>
-  <si>
-    <t>0.56s</t>
-  </si>
-  <si>
-    <t>0.00s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:16 pm</t>
-  </si>
-  <si>
-    <t>0.35s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:17 pm</t>
-  </si>
-  <si>
-    <t>0.38s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:21:18 pm</t>
-  </si>
-  <si>
-    <t>0.41s</t>
-  </si>
-  <si>
-    <t>0.27s</t>
+    <t>0.31s</t>
   </si>
 </sst>
 </file>
@@ -15483,7 +15474,7 @@
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>1337</v>
+        <v>1327</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15763,7 +15754,7 @@
         <v>9</v>
       </c>
       <c r="C82" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -16177,13 +16168,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B112" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" t="s">
         <v>1339</v>
-      </c>
-      <c r="B112" t="s">
-        <v>9</v>
-      </c>
-      <c r="C112" t="s">
-        <v>1340</v>
       </c>
       <c r="D112" t="s">
         <v>35</v>
@@ -16191,7 +16182,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B113" t="s">
         <v>9</v>
@@ -16205,7 +16196,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B114" t="s">
         <v>9</v>
@@ -16219,7 +16210,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B115" t="s">
         <v>9</v>
@@ -16233,7 +16224,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B116" t="s">
         <v>9</v>
@@ -16247,7 +16238,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B117" t="s">
         <v>9</v>
@@ -16261,7 +16252,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B118" t="s">
         <v>9</v>
@@ -16275,7 +16266,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B119" t="s">
         <v>9</v>
@@ -16289,7 +16280,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B120" t="s">
         <v>9</v>
@@ -16303,7 +16294,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B121" t="s">
         <v>9</v>
@@ -16317,7 +16308,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B122" t="s">
         <v>9</v>
@@ -16331,7 +16322,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B123" t="s">
         <v>9</v>
@@ -16345,7 +16336,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B124" t="s">
         <v>9</v>
@@ -16359,7 +16350,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B125" t="s">
         <v>9</v>
@@ -16373,7 +16364,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B126" t="s">
         <v>9</v>
@@ -16387,7 +16378,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -16401,7 +16392,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -16415,7 +16406,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -16429,7 +16420,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -16443,7 +16434,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -16457,7 +16448,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -16471,7 +16462,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -16485,7 +16476,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -16499,13 +16490,13 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
       </c>
       <c r="C135" t="s">
-        <v>1341</v>
+        <v>1317</v>
       </c>
       <c r="D135" t="s">
         <v>35</v>
@@ -16513,7 +16504,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -16527,13 +16518,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B137" t="s">
         <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="D137" t="s">
         <v>35</v>
@@ -16541,7 +16532,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -16555,7 +16546,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -16569,7 +16560,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -16583,7 +16574,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -16597,7 +16588,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -16611,7 +16602,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -16625,7 +16616,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -16639,7 +16630,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -16653,7 +16644,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -16667,7 +16658,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -16681,7 +16672,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -16695,7 +16686,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -16709,7 +16700,7 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -16723,7 +16714,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -16737,7 +16728,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -16751,7 +16742,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -16765,7 +16756,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -16779,7 +16770,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -16793,7 +16784,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -16807,7 +16798,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -16821,7 +16812,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -16835,7 +16826,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -16849,7 +16840,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -16863,7 +16854,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -16877,7 +16868,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -16891,7 +16882,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -16905,7 +16896,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -16919,7 +16910,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -16933,7 +16924,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>1342</v>
+        <v>1338</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -16947,13 +16938,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
       </c>
       <c r="C167" t="s">
-        <v>1343</v>
+        <v>1339</v>
       </c>
       <c r="D167" t="s">
         <v>35</v>
@@ -16961,7 +16952,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -16975,7 +16966,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -16989,7 +16980,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -17003,7 +16994,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -17017,7 +17008,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -17031,7 +17022,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -17045,7 +17036,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -17059,7 +17050,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B175" t="s">
         <v>9</v>
@@ -17073,7 +17064,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -17087,7 +17078,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -17101,7 +17092,7 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -17115,7 +17106,7 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -17129,7 +17120,7 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -17143,7 +17134,7 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -17157,7 +17148,7 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -17171,7 +17162,7 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -17185,7 +17176,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -17199,7 +17190,7 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -17213,7 +17204,7 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -17227,7 +17218,7 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -17241,7 +17232,7 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -17255,7 +17246,7 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -17269,7 +17260,7 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -17283,7 +17274,7 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -17297,13 +17288,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
       </c>
       <c r="C192" t="s">
-        <v>1345</v>
+        <v>1337</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17311,7 +17302,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17325,7 +17316,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17339,7 +17330,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17353,7 +17344,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17367,7 +17358,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17381,7 +17372,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17395,7 +17386,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17409,7 +17400,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17423,7 +17414,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17437,7 +17428,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17451,7 +17442,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17465,7 +17456,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17479,7 +17470,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17493,7 +17484,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17507,7 +17498,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17521,7 +17512,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17535,7 +17526,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17549,7 +17540,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17563,7 +17554,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17577,7 +17568,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17591,7 +17582,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17605,7 +17596,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17619,7 +17610,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17633,7 +17624,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17647,7 +17638,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17661,7 +17652,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17675,7 +17666,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17689,7 +17680,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17703,7 +17694,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17717,13 +17708,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
       </c>
       <c r="C222" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="D222" t="s">
         <v>35</v>
@@ -17731,7 +17722,7 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -17745,7 +17736,7 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -17759,7 +17750,7 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -17773,7 +17764,7 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -17787,7 +17778,7 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -17801,7 +17792,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -17815,7 +17806,7 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -17829,7 +17820,7 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -17843,7 +17834,7 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -17857,7 +17848,7 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>
@@ -17871,7 +17862,7 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B233" t="s">
         <v>9</v>
@@ -17885,7 +17876,7 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B234" t="s">
         <v>9</v>
@@ -17899,7 +17890,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B235" t="s">
         <v>9</v>
@@ -17913,7 +17904,7 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B236" t="s">
         <v>9</v>
@@ -17927,13 +17918,13 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B237" t="s">
         <v>9</v>
       </c>
       <c r="C237" t="s">
-        <v>1341</v>
+        <v>1317</v>
       </c>
       <c r="D237" t="s">
         <v>35</v>
@@ -17941,7 +17932,7 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B238" t="s">
         <v>9</v>
@@ -17955,7 +17946,7 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B239" t="s">
         <v>9</v>
@@ -17969,7 +17960,7 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B240" t="s">
         <v>9</v>
@@ -17983,7 +17974,7 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B241" t="s">
         <v>9</v>
@@ -17997,7 +17988,7 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B242" t="s">
         <v>9</v>
@@ -18011,7 +18002,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B243" t="s">
         <v>9</v>
@@ -18025,7 +18016,7 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B244" t="s">
         <v>9</v>
@@ -18039,7 +18030,7 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B245" t="s">
         <v>9</v>
@@ -18053,7 +18044,7 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B246" t="s">
         <v>9</v>
@@ -18067,13 +18058,13 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B247" t="s">
         <v>9</v>
       </c>
       <c r="C247" t="s">
-        <v>1345</v>
+        <v>1337</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18081,7 +18072,7 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B248" t="s">
         <v>9</v>
@@ -18095,7 +18086,7 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B249" t="s">
         <v>9</v>
@@ -18109,7 +18100,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B250" t="s">
         <v>9</v>
@@ -18123,7 +18114,7 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B251" t="s">
         <v>9</v>
@@ -18137,7 +18128,7 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B252" t="s">
         <v>9</v>
@@ -18151,7 +18142,7 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B253" t="s">
         <v>9</v>
@@ -18165,7 +18156,7 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B254" t="s">
         <v>9</v>
@@ -18179,7 +18170,7 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B255" t="s">
         <v>9</v>
@@ -18193,7 +18184,7 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B256" t="s">
         <v>9</v>
@@ -18207,7 +18198,7 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B257" t="s">
         <v>9</v>
@@ -18221,7 +18212,7 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B258" t="s">
         <v>9</v>
@@ -18235,7 +18226,7 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B259" t="s">
         <v>9</v>
@@ -18249,7 +18240,7 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B260" t="s">
         <v>9</v>
@@ -18263,7 +18254,7 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B261" t="s">
         <v>9</v>
@@ -18277,7 +18268,7 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B262" t="s">
         <v>9</v>
@@ -18291,7 +18282,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B263" t="s">
         <v>9</v>
@@ -18305,7 +18296,7 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B264" t="s">
         <v>9</v>
@@ -18319,7 +18310,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B265" t="s">
         <v>9</v>
@@ -18333,7 +18324,7 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B266" t="s">
         <v>9</v>
@@ -18347,7 +18338,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B267" t="s">
         <v>9</v>
@@ -18361,7 +18352,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B268" t="s">
         <v>9</v>
@@ -18375,7 +18366,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B269" t="s">
         <v>9</v>
@@ -18389,7 +18380,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B270" t="s">
         <v>9</v>
@@ -18403,7 +18394,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="B271" t="s">
         <v>9</v>
@@ -18417,13 +18408,13 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B272" t="s">
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1347</v>
+        <v>1344</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18431,7 +18422,7 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B273" t="s">
         <v>9</v>
@@ -18445,7 +18436,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B274" t="s">
         <v>9</v>
@@ -18459,7 +18450,7 @@
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B275" t="s">
         <v>9</v>
@@ -18473,7 +18464,7 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B276" t="s">
         <v>9</v>
@@ -18487,7 +18478,7 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B277" t="s">
         <v>9</v>
@@ -18501,7 +18492,7 @@
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B278" t="s">
         <v>9</v>
@@ -18515,7 +18506,7 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B279" t="s">
         <v>9</v>
@@ -18529,7 +18520,7 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B280" t="s">
         <v>9</v>
@@ -18543,7 +18534,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B281" t="s">
         <v>9</v>
@@ -18557,7 +18548,7 @@
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B282" t="s">
         <v>9</v>
@@ -18571,7 +18562,7 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B283" t="s">
         <v>9</v>
@@ -18585,7 +18576,7 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B284" t="s">
         <v>9</v>
@@ -18599,7 +18590,7 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B285" t="s">
         <v>9</v>
@@ -18613,7 +18604,7 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B286" t="s">
         <v>9</v>
@@ -18627,7 +18618,7 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B287" t="s">
         <v>9</v>
@@ -18641,7 +18632,7 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B288" t="s">
         <v>9</v>
@@ -18655,7 +18646,7 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B289" t="s">
         <v>9</v>
@@ -18669,7 +18660,7 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B290" t="s">
         <v>9</v>
@@ -18683,7 +18674,7 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B291" t="s">
         <v>9</v>
@@ -18697,7 +18688,7 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B292" t="s">
         <v>9</v>
@@ -18711,7 +18702,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B293" t="s">
         <v>9</v>
@@ -18725,7 +18716,7 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B294" t="s">
         <v>9</v>
@@ -18739,7 +18730,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B295" t="s">
         <v>9</v>
@@ -18753,7 +18744,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B296" t="s">
         <v>9</v>
@@ -18767,13 +18758,13 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B297" t="s">
         <v>9</v>
       </c>
       <c r="C297" t="s">
-        <v>1348</v>
+        <v>1345</v>
       </c>
       <c r="D297" t="s">
         <v>35</v>
@@ -18781,7 +18772,7 @@
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B298" t="s">
         <v>9</v>
@@ -18795,7 +18786,7 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B299" t="s">
         <v>9</v>
@@ -18809,7 +18800,7 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B300" t="s">
         <v>9</v>
@@ -18823,7 +18814,7 @@
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B301" t="s">
         <v>9</v>
@@ -18837,7 +18828,7 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B302" t="s">
         <v>9</v>
@@ -18851,7 +18842,7 @@
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B303" t="s">
         <v>9</v>
@@ -18865,7 +18856,7 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B304" t="s">
         <v>9</v>
@@ -18879,7 +18870,7 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B305" t="s">
         <v>9</v>
@@ -18893,7 +18884,7 @@
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B306" t="s">
         <v>9</v>
@@ -18907,7 +18898,7 @@
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B307" t="s">
         <v>9</v>
@@ -18921,7 +18912,7 @@
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B308" t="s">
         <v>9</v>
@@ -18935,7 +18926,7 @@
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B309" t="s">
         <v>9</v>
@@ -18949,7 +18940,7 @@
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B310" t="s">
         <v>9</v>
@@ -18963,7 +18954,7 @@
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>7</v>
+        <v>1343</v>
       </c>
       <c r="B311" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Update Selenium test suite for 310/310 passed test cases on production build
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1354">
   <si>
     <t>Metric</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 6:32:41 pm</t>
+    <t>28/7/2026, 9:19:19 pm</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>39.91 seconds</t>
+    <t>53.42 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,109 +3949,133 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 6:32:05 pm</t>
+    <t>28/7/2026, 9:18:36 pm</t>
+  </si>
+  <si>
+    <t>2.39s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:39 pm</t>
+  </si>
+  <si>
+    <t>2.79s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:42 pm</t>
+  </si>
+  <si>
+    <t>2.67s</t>
+  </si>
+  <si>
+    <t>0.15s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:45 pm</t>
+  </si>
+  <si>
+    <t>2.94s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:50 pm</t>
+  </si>
+  <si>
+    <t>5.82s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:53 pm</t>
+  </si>
+  <si>
+    <t>2.42s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:55 pm</t>
+  </si>
+  <si>
+    <t>2.37s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:18:57 pm</t>
+  </si>
+  <si>
+    <t>2.13s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:00 pm</t>
   </si>
   <si>
     <t>2.06s</t>
   </si>
   <si>
-    <t>28/7/2026, 6:32:07 pm</t>
+    <t>28/7/2026, 9:19:02 pm</t>
   </si>
   <si>
     <t>2.85s</t>
   </si>
   <si>
-    <t>28/7/2026, 6:32:10 pm</t>
-  </si>
-  <si>
-    <t>2.43s</t>
-  </si>
-  <si>
-    <t>0.15s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:12 pm</t>
-  </si>
-  <si>
-    <t>2.48s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:15 pm</t>
-  </si>
-  <si>
-    <t>2.56s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:17 pm</t>
-  </si>
-  <si>
-    <t>2.51s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:20 pm</t>
-  </si>
-  <si>
-    <t>2.71s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:22 pm</t>
-  </si>
-  <si>
-    <t>2.18s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:25 pm</t>
-  </si>
-  <si>
-    <t>2.20s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:28 pm</t>
-  </si>
-  <si>
-    <t>2.93s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:31 pm</t>
-  </si>
-  <si>
-    <t>2.46s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:33 pm</t>
-  </si>
-  <si>
-    <t>2.21s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:36 pm</t>
+    <t>28/7/2026, 9:19:06 pm</t>
+  </si>
+  <si>
+    <t>3.96s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:10 pm</t>
+  </si>
+  <si>
+    <t>3.29s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:12 pm</t>
+  </si>
+  <si>
+    <t>2.30s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:13 pm</t>
+  </si>
+  <si>
+    <t>0.51s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:14 pm</t>
+  </si>
+  <si>
+    <t>0.63s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:15 pm</t>
+  </si>
+  <si>
+    <t>0.52s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:16 pm</t>
+  </si>
+  <si>
+    <t>0.45s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:19:17 pm</t>
+  </si>
+  <si>
+    <t>0.43s</t>
   </si>
   <si>
     <t>0.37s</t>
   </si>
   <si>
-    <t>28/7/2026, 6:32:37 pm</t>
-  </si>
-  <si>
-    <t>0.38s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:38 pm</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:39 pm</t>
-  </si>
-  <si>
-    <t>0.36s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 6:32:40 pm</t>
+    <t>28/7/2026, 9:19:18 pm</t>
+  </si>
+  <si>
+    <t>0.34s</t>
   </si>
   <si>
     <t>0.40s</t>
   </si>
   <si>
-    <t>0.31s</t>
+    <t>0.47s</t>
+  </si>
+  <si>
+    <t>0.00s</t>
   </si>
 </sst>
 </file>
@@ -15474,7 +15498,7 @@
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>1327</v>
+        <v>1337</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15748,13 +15772,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B82" t="s">
         <v>9</v>
       </c>
       <c r="C82" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -15762,7 +15786,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
@@ -15776,7 +15800,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -15790,7 +15814,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -15804,7 +15828,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -15818,7 +15842,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B87" t="s">
         <v>9</v>
@@ -15832,7 +15856,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B88" t="s">
         <v>9</v>
@@ -15846,7 +15870,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -15860,7 +15884,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -15874,7 +15898,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -15888,7 +15912,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -15902,7 +15926,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B93" t="s">
         <v>9</v>
@@ -15916,7 +15940,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B94" t="s">
         <v>9</v>
@@ -15930,7 +15954,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B95" t="s">
         <v>9</v>
@@ -15944,7 +15968,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B96" t="s">
         <v>9</v>
@@ -15958,7 +15982,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -15972,7 +15996,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B98" t="s">
         <v>9</v>
@@ -15986,7 +16010,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -16000,7 +16024,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B100" t="s">
         <v>9</v>
@@ -16014,7 +16038,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -16028,7 +16052,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B102" t="s">
         <v>9</v>
@@ -16042,7 +16066,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B103" t="s">
         <v>9</v>
@@ -16056,7 +16080,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B104" t="s">
         <v>9</v>
@@ -16070,7 +16094,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -16084,7 +16108,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B106" t="s">
         <v>9</v>
@@ -16098,7 +16122,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
@@ -16112,7 +16136,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B108" t="s">
         <v>9</v>
@@ -16126,7 +16150,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B109" t="s">
         <v>9</v>
@@ -16140,7 +16164,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B110" t="s">
         <v>9</v>
@@ -16154,7 +16178,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -16168,13 +16192,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B112" t="s">
         <v>9</v>
       </c>
       <c r="C112" t="s">
-        <v>1339</v>
+        <v>1341</v>
       </c>
       <c r="D112" t="s">
         <v>35</v>
@@ -16182,7 +16206,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B113" t="s">
         <v>9</v>
@@ -16196,7 +16220,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B114" t="s">
         <v>9</v>
@@ -16210,7 +16234,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B115" t="s">
         <v>9</v>
@@ -16224,7 +16248,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B116" t="s">
         <v>9</v>
@@ -16238,7 +16262,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B117" t="s">
         <v>9</v>
@@ -16252,7 +16276,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B118" t="s">
         <v>9</v>
@@ -16266,7 +16290,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B119" t="s">
         <v>9</v>
@@ -16280,7 +16304,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B120" t="s">
         <v>9</v>
@@ -16294,7 +16318,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B121" t="s">
         <v>9</v>
@@ -16308,7 +16332,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B122" t="s">
         <v>9</v>
@@ -16322,7 +16346,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B123" t="s">
         <v>9</v>
@@ -16336,7 +16360,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B124" t="s">
         <v>9</v>
@@ -16350,7 +16374,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B125" t="s">
         <v>9</v>
@@ -16364,7 +16388,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B126" t="s">
         <v>9</v>
@@ -16378,7 +16402,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -16392,7 +16416,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -16406,7 +16430,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -16420,7 +16444,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -16434,7 +16458,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -16448,7 +16472,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -16462,7 +16486,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -16476,7 +16500,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -16490,7 +16514,7 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
@@ -16504,7 +16528,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -16518,13 +16542,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B137" t="s">
         <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>1339</v>
+        <v>1343</v>
       </c>
       <c r="D137" t="s">
         <v>35</v>
@@ -16532,7 +16556,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -16546,7 +16570,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -16560,7 +16584,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -16574,7 +16598,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -16588,7 +16612,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -16602,7 +16626,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -16616,7 +16640,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -16630,7 +16654,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -16644,7 +16668,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -16658,7 +16682,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -16672,7 +16696,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -16686,7 +16710,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -16700,7 +16724,7 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -16714,7 +16738,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -16728,7 +16752,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -16742,7 +16766,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -16756,7 +16780,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -16770,7 +16794,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -16784,7 +16808,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -16798,7 +16822,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -16812,7 +16836,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -16826,7 +16850,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -16840,7 +16864,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -16854,7 +16878,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -16868,7 +16892,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -16882,7 +16906,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -16896,7 +16920,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -16910,7 +16934,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -16924,7 +16948,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -16938,13 +16962,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
       </c>
       <c r="C167" t="s">
-        <v>1339</v>
+        <v>1345</v>
       </c>
       <c r="D167" t="s">
         <v>35</v>
@@ -16952,7 +16976,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -16966,7 +16990,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -16980,7 +17004,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -16994,7 +17018,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -17008,7 +17032,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -17022,7 +17046,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -17036,7 +17060,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -17050,7 +17074,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B175" t="s">
         <v>9</v>
@@ -17064,7 +17088,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -17078,7 +17102,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -17092,7 +17116,7 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -17106,7 +17130,7 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -17120,7 +17144,7 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -17134,7 +17158,7 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -17148,7 +17172,7 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -17162,7 +17186,7 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -17176,7 +17200,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -17190,7 +17214,7 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -17204,7 +17228,7 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -17218,7 +17242,7 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -17232,7 +17256,7 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -17246,7 +17270,7 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -17260,7 +17284,7 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -17274,7 +17298,7 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -17288,13 +17312,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B192" t="s">
         <v>9</v>
       </c>
       <c r="C192" t="s">
-        <v>1337</v>
+        <v>1347</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17302,7 +17326,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17316,7 +17340,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17330,7 +17354,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17344,7 +17368,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17358,7 +17382,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17372,7 +17396,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17386,7 +17410,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17400,7 +17424,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17414,7 +17438,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17428,7 +17452,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17442,7 +17466,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17456,7 +17480,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17470,7 +17494,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17484,7 +17508,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17498,7 +17522,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17512,7 +17536,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17526,7 +17550,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17540,7 +17564,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17554,7 +17578,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17568,7 +17592,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17582,7 +17606,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17596,7 +17620,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17610,7 +17634,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17624,7 +17648,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17638,7 +17662,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17652,7 +17676,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17666,7 +17690,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17680,7 +17704,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17694,7 +17718,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1340</v>
+        <v>1346</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17708,13 +17732,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
       </c>
       <c r="C222" t="s">
-        <v>1342</v>
+        <v>1348</v>
       </c>
       <c r="D222" t="s">
         <v>35</v>
@@ -17722,7 +17746,7 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -17736,7 +17760,7 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -17750,7 +17774,7 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -17764,7 +17788,7 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -17778,7 +17802,7 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -17792,7 +17816,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -17806,7 +17830,7 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -17820,7 +17844,7 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -17834,7 +17858,7 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -17848,7 +17872,7 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>
@@ -17862,7 +17886,7 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B233" t="s">
         <v>9</v>
@@ -17876,7 +17900,7 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B234" t="s">
         <v>9</v>
@@ -17890,7 +17914,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B235" t="s">
         <v>9</v>
@@ -17904,7 +17928,7 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B236" t="s">
         <v>9</v>
@@ -17918,7 +17942,7 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B237" t="s">
         <v>9</v>
@@ -17932,7 +17956,7 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B238" t="s">
         <v>9</v>
@@ -17946,7 +17970,7 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B239" t="s">
         <v>9</v>
@@ -17960,7 +17984,7 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B240" t="s">
         <v>9</v>
@@ -17974,7 +17998,7 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B241" t="s">
         <v>9</v>
@@ -17988,7 +18012,7 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B242" t="s">
         <v>9</v>
@@ -18002,7 +18026,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B243" t="s">
         <v>9</v>
@@ -18016,7 +18040,7 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B244" t="s">
         <v>9</v>
@@ -18030,7 +18054,7 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B245" t="s">
         <v>9</v>
@@ -18044,7 +18068,7 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="B246" t="s">
         <v>9</v>
@@ -18058,13 +18082,13 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B247" t="s">
         <v>9</v>
       </c>
       <c r="C247" t="s">
-        <v>1337</v>
+        <v>1350</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18072,7 +18096,7 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B248" t="s">
         <v>9</v>
@@ -18086,7 +18110,7 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B249" t="s">
         <v>9</v>
@@ -18100,7 +18124,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B250" t="s">
         <v>9</v>
@@ -18114,7 +18138,7 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B251" t="s">
         <v>9</v>
@@ -18128,7 +18152,7 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B252" t="s">
         <v>9</v>
@@ -18142,7 +18166,7 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B253" t="s">
         <v>9</v>
@@ -18156,7 +18180,7 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B254" t="s">
         <v>9</v>
@@ -18170,7 +18194,7 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B255" t="s">
         <v>9</v>
@@ -18184,7 +18208,7 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B256" t="s">
         <v>9</v>
@@ -18198,7 +18222,7 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B257" t="s">
         <v>9</v>
@@ -18212,7 +18236,7 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B258" t="s">
         <v>9</v>
@@ -18226,7 +18250,7 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B259" t="s">
         <v>9</v>
@@ -18240,7 +18264,7 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B260" t="s">
         <v>9</v>
@@ -18254,7 +18278,7 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B261" t="s">
         <v>9</v>
@@ -18268,7 +18292,7 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B262" t="s">
         <v>9</v>
@@ -18282,7 +18306,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B263" t="s">
         <v>9</v>
@@ -18296,7 +18320,7 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B264" t="s">
         <v>9</v>
@@ -18310,7 +18334,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B265" t="s">
         <v>9</v>
@@ -18324,7 +18348,7 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B266" t="s">
         <v>9</v>
@@ -18338,7 +18362,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B267" t="s">
         <v>9</v>
@@ -18352,7 +18376,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B268" t="s">
         <v>9</v>
@@ -18366,7 +18390,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B269" t="s">
         <v>9</v>
@@ -18380,7 +18404,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B270" t="s">
         <v>9</v>
@@ -18394,7 +18418,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1341</v>
+        <v>1349</v>
       </c>
       <c r="B271" t="s">
         <v>9</v>
@@ -18408,13 +18432,13 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B272" t="s">
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1344</v>
+        <v>1351</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18422,7 +18446,7 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B273" t="s">
         <v>9</v>
@@ -18436,7 +18460,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B274" t="s">
         <v>9</v>
@@ -18450,7 +18474,7 @@
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B275" t="s">
         <v>9</v>
@@ -18464,7 +18488,7 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B276" t="s">
         <v>9</v>
@@ -18478,7 +18502,7 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B277" t="s">
         <v>9</v>
@@ -18492,7 +18516,7 @@
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B278" t="s">
         <v>9</v>
@@ -18506,7 +18530,7 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B279" t="s">
         <v>9</v>
@@ -18520,7 +18544,7 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B280" t="s">
         <v>9</v>
@@ -18534,7 +18558,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B281" t="s">
         <v>9</v>
@@ -18548,7 +18572,7 @@
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B282" t="s">
         <v>9</v>
@@ -18562,7 +18586,7 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B283" t="s">
         <v>9</v>
@@ -18576,7 +18600,7 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B284" t="s">
         <v>9</v>
@@ -18590,7 +18614,7 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B285" t="s">
         <v>9</v>
@@ -18604,7 +18628,7 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B286" t="s">
         <v>9</v>
@@ -18618,7 +18642,7 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B287" t="s">
         <v>9</v>
@@ -18632,7 +18656,7 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B288" t="s">
         <v>9</v>
@@ -18646,7 +18670,7 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B289" t="s">
         <v>9</v>
@@ -18660,7 +18684,7 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B290" t="s">
         <v>9</v>
@@ -18674,7 +18698,7 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B291" t="s">
         <v>9</v>
@@ -18688,7 +18712,7 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B292" t="s">
         <v>9</v>
@@ -18702,7 +18726,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B293" t="s">
         <v>9</v>
@@ -18716,7 +18740,7 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B294" t="s">
         <v>9</v>
@@ -18730,7 +18754,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B295" t="s">
         <v>9</v>
@@ -18744,7 +18768,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B296" t="s">
         <v>9</v>
@@ -18758,13 +18782,13 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B297" t="s">
         <v>9</v>
       </c>
       <c r="C297" t="s">
-        <v>1345</v>
+        <v>1352</v>
       </c>
       <c r="D297" t="s">
         <v>35</v>
@@ -18772,7 +18796,7 @@
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B298" t="s">
         <v>9</v>
@@ -18786,7 +18810,7 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B299" t="s">
         <v>9</v>
@@ -18800,7 +18824,7 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B300" t="s">
         <v>9</v>
@@ -18814,7 +18838,7 @@
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B301" t="s">
         <v>9</v>
@@ -18828,13 +18852,13 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B302" t="s">
         <v>9</v>
       </c>
       <c r="C302" t="s">
-        <v>1317</v>
+        <v>1353</v>
       </c>
       <c r="D302" t="s">
         <v>35</v>
@@ -18842,7 +18866,7 @@
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B303" t="s">
         <v>9</v>
@@ -18856,7 +18880,7 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B304" t="s">
         <v>9</v>
@@ -18870,7 +18894,7 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B305" t="s">
         <v>9</v>
@@ -18884,7 +18908,7 @@
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B306" t="s">
         <v>9</v>
@@ -18898,7 +18922,7 @@
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B307" t="s">
         <v>9</v>
@@ -18912,7 +18936,7 @@
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B308" t="s">
         <v>9</v>
@@ -18926,7 +18950,7 @@
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B309" t="s">
         <v>9</v>
@@ -18940,7 +18964,7 @@
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B310" t="s">
         <v>9</v>
@@ -18954,7 +18978,7 @@
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>1343</v>
+        <v>7</v>
       </c>
       <c r="B311" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Update Selenium test reports for 310/310 passed test cases
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1352">
   <si>
     <t>Metric</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 9:19:19 pm</t>
+    <t>28/7/2026, 9:39:49 pm</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>53.42 seconds</t>
+    <t>41.28 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,133 +3949,127 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 9:18:36 pm</t>
-  </si>
-  <si>
-    <t>2.39s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:39 pm</t>
-  </si>
-  <si>
-    <t>2.79s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:42 pm</t>
-  </si>
-  <si>
-    <t>2.67s</t>
+    <t>28/7/2026, 9:39:11 pm</t>
+  </si>
+  <si>
+    <t>2.02s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:14 pm</t>
+  </si>
+  <si>
+    <t>2.83s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:17 pm</t>
+  </si>
+  <si>
+    <t>2.55s</t>
   </si>
   <si>
     <t>0.15s</t>
   </si>
   <si>
-    <t>28/7/2026, 9:18:45 pm</t>
-  </si>
-  <si>
-    <t>2.94s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:50 pm</t>
-  </si>
-  <si>
-    <t>5.82s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:53 pm</t>
-  </si>
-  <si>
-    <t>2.42s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:55 pm</t>
-  </si>
-  <si>
-    <t>2.37s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:18:57 pm</t>
-  </si>
-  <si>
-    <t>2.13s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:00 pm</t>
-  </si>
-  <si>
-    <t>2.06s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:02 pm</t>
-  </si>
-  <si>
-    <t>2.85s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:06 pm</t>
-  </si>
-  <si>
-    <t>3.96s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:10 pm</t>
-  </si>
-  <si>
-    <t>3.29s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:12 pm</t>
-  </si>
-  <si>
-    <t>2.30s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:13 pm</t>
-  </si>
-  <si>
-    <t>0.51s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:14 pm</t>
-  </si>
-  <si>
-    <t>0.63s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:15 pm</t>
-  </si>
-  <si>
-    <t>0.52s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:16 pm</t>
-  </si>
-  <si>
-    <t>0.45s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:17 pm</t>
+    <t>28/7/2026, 9:39:20 pm</t>
+  </si>
+  <si>
+    <t>2.75s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:21 pm</t>
+  </si>
+  <si>
+    <t>1.26s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:23 pm</t>
+  </si>
+  <si>
+    <t>2.35s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:26 pm</t>
+  </si>
+  <si>
+    <t>2.43s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:30 pm</t>
+  </si>
+  <si>
+    <t>4.52s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:32 pm</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:35 pm</t>
+  </si>
+  <si>
+    <t>2.87s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:38 pm</t>
+  </si>
+  <si>
+    <t>2.32s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:40 pm</t>
+  </si>
+  <si>
+    <t>2.63s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:43 pm</t>
+  </si>
+  <si>
+    <t>2.24s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:44 pm</t>
+  </si>
+  <si>
+    <t>0.53s</t>
+  </si>
+  <si>
+    <t>0.00s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:45 pm</t>
+  </si>
+  <si>
+    <t>0.78s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:46 pm</t>
   </si>
   <si>
     <t>0.43s</t>
   </si>
   <si>
-    <t>0.37s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:19:18 pm</t>
-  </si>
-  <si>
-    <t>0.34s</t>
-  </si>
-  <si>
-    <t>0.40s</t>
-  </si>
-  <si>
-    <t>0.47s</t>
-  </si>
-  <si>
-    <t>0.00s</t>
+    <t>28/7/2026, 9:39:47 pm</t>
+  </si>
+  <si>
+    <t>0.77s</t>
+  </si>
+  <si>
+    <t>0.41s</t>
+  </si>
+  <si>
+    <t>28/7/2026, 9:39:48 pm</t>
+  </si>
+  <si>
+    <t>0.30s</t>
+  </si>
+  <si>
+    <t>0.35s</t>
+  </si>
+  <si>
+    <t>0.33s</t>
+  </si>
+  <si>
+    <t>0.24s</t>
   </si>
 </sst>
 </file>
@@ -15078,7 +15072,7 @@
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>1329</v>
+        <v>1312</v>
       </c>
       <c r="D32" t="s">
         <v>35</v>
@@ -15086,13 +15080,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
         <v>1330</v>
-      </c>
-      <c r="B33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1331</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -15100,7 +15094,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -15114,7 +15108,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
@@ -15128,7 +15122,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
@@ -15142,7 +15136,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -15156,7 +15150,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -15170,7 +15164,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -15184,7 +15178,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -15198,13 +15192,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
         <v>1332</v>
-      </c>
-      <c r="B41" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1333</v>
       </c>
       <c r="D41" t="s">
         <v>35</v>
@@ -15212,13 +15206,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
         <v>1334</v>
-      </c>
-      <c r="B42" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" t="s">
-        <v>1335</v>
       </c>
       <c r="D42" t="s">
         <v>35</v>
@@ -15226,7 +15220,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -15240,7 +15234,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -15254,7 +15248,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -15268,7 +15262,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -15282,7 +15276,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -15296,7 +15290,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -15310,7 +15304,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -15324,7 +15318,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -15338,7 +15332,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -15352,7 +15346,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -15366,7 +15360,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -15380,7 +15374,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -15394,7 +15388,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -15408,7 +15402,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -15422,7 +15416,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B57" t="s">
         <v>9</v>
@@ -15436,7 +15430,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -15450,7 +15444,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
@@ -15464,7 +15458,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
@@ -15478,7 +15472,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B61" t="s">
         <v>9</v>
@@ -15492,13 +15486,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
         <v>1336</v>
-      </c>
-      <c r="B62" t="s">
-        <v>9</v>
-      </c>
-      <c r="C62" t="s">
-        <v>1337</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15506,7 +15500,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -15520,7 +15514,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
@@ -15534,7 +15528,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -15548,7 +15542,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B66" t="s">
         <v>9</v>
@@ -15562,7 +15556,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -15576,7 +15570,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -15590,7 +15584,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -15604,7 +15598,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
@@ -15618,7 +15612,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B71" t="s">
         <v>9</v>
@@ -15632,7 +15626,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B72" t="s">
         <v>9</v>
@@ -15646,7 +15640,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
@@ -15660,7 +15654,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B74" t="s">
         <v>9</v>
@@ -15674,7 +15668,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B75" t="s">
         <v>9</v>
@@ -15688,7 +15682,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -15702,7 +15696,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
@@ -15716,7 +15710,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
@@ -15730,7 +15724,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
@@ -15744,7 +15738,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -15758,7 +15752,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
@@ -15772,13 +15766,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
         <v>1338</v>
-      </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
-      <c r="C82" t="s">
-        <v>1339</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -15786,13 +15780,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
       </c>
       <c r="C83" t="s">
-        <v>1317</v>
+        <v>1339</v>
       </c>
       <c r="D83" t="s">
         <v>35</v>
@@ -15800,7 +15794,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -15814,7 +15808,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -15828,7 +15822,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -15842,7 +15836,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B87" t="s">
         <v>9</v>
@@ -15856,7 +15850,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B88" t="s">
         <v>9</v>
@@ -15870,7 +15864,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -15884,7 +15878,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -15898,7 +15892,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -15912,7 +15906,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -15926,7 +15920,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B93" t="s">
         <v>9</v>
@@ -15940,7 +15934,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B94" t="s">
         <v>9</v>
@@ -15954,7 +15948,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B95" t="s">
         <v>9</v>
@@ -15968,7 +15962,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B96" t="s">
         <v>9</v>
@@ -15982,7 +15976,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -15996,7 +15990,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B98" t="s">
         <v>9</v>
@@ -16010,7 +16004,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -16024,7 +16018,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B100" t="s">
         <v>9</v>
@@ -16038,7 +16032,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -16052,7 +16046,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B102" t="s">
         <v>9</v>
@@ -16066,7 +16060,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B103" t="s">
         <v>9</v>
@@ -16080,7 +16074,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B104" t="s">
         <v>9</v>
@@ -16094,7 +16088,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -16108,7 +16102,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B106" t="s">
         <v>9</v>
@@ -16122,7 +16116,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
@@ -16136,7 +16130,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B108" t="s">
         <v>9</v>
@@ -16150,7 +16144,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B109" t="s">
         <v>9</v>
@@ -16164,7 +16158,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B110" t="s">
         <v>9</v>
@@ -16178,7 +16172,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -17312,13 +17306,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B192" t="s">
+        <v>9</v>
+      </c>
+      <c r="C192" t="s">
         <v>1346</v>
-      </c>
-      <c r="B192" t="s">
-        <v>9</v>
-      </c>
-      <c r="C192" t="s">
-        <v>1347</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17326,7 +17320,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17340,7 +17334,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17354,7 +17348,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17368,7 +17362,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17382,7 +17376,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17396,7 +17390,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17410,7 +17404,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17424,7 +17418,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17438,7 +17432,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17452,7 +17446,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17466,7 +17460,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17480,7 +17474,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17494,7 +17488,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17508,7 +17502,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17522,7 +17516,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17536,7 +17530,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17550,7 +17544,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17564,7 +17558,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17578,7 +17572,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17592,7 +17586,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17606,7 +17600,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17620,7 +17614,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17634,7 +17628,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17648,7 +17642,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17662,7 +17656,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17676,7 +17670,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17690,7 +17684,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17704,7 +17698,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17718,7 +17712,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17732,7 +17726,7 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
@@ -17746,7 +17740,7 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -17760,7 +17754,7 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -17774,7 +17768,7 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -17788,7 +17782,7 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -17802,7 +17796,7 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -17816,7 +17810,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -17830,7 +17824,7 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -17844,7 +17838,7 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -17858,7 +17852,7 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -17872,7 +17866,7 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>
@@ -17886,7 +17880,7 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B233" t="s">
         <v>9</v>
@@ -17900,7 +17894,7 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B234" t="s">
         <v>9</v>
@@ -17914,7 +17908,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B235" t="s">
         <v>9</v>
@@ -17928,7 +17922,7 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B236" t="s">
         <v>9</v>
@@ -17942,7 +17936,7 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B237" t="s">
         <v>9</v>
@@ -17956,7 +17950,7 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B238" t="s">
         <v>9</v>
@@ -17970,7 +17964,7 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B239" t="s">
         <v>9</v>
@@ -17984,7 +17978,7 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B240" t="s">
         <v>9</v>
@@ -17998,7 +17992,7 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B241" t="s">
         <v>9</v>
@@ -18012,7 +18006,7 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B242" t="s">
         <v>9</v>
@@ -18026,7 +18020,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B243" t="s">
         <v>9</v>
@@ -18040,7 +18034,7 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B244" t="s">
         <v>9</v>
@@ -18054,7 +18048,7 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B245" t="s">
         <v>9</v>
@@ -18068,7 +18062,7 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B246" t="s">
         <v>9</v>
@@ -18082,13 +18076,13 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B247" t="s">
+        <v>9</v>
+      </c>
+      <c r="C247" t="s">
         <v>1349</v>
-      </c>
-      <c r="B247" t="s">
-        <v>9</v>
-      </c>
-      <c r="C247" t="s">
-        <v>1350</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18096,7 +18090,7 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B248" t="s">
         <v>9</v>
@@ -18110,7 +18104,7 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B249" t="s">
         <v>9</v>
@@ -18124,7 +18118,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B250" t="s">
         <v>9</v>
@@ -18138,7 +18132,7 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B251" t="s">
         <v>9</v>
@@ -18152,7 +18146,7 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B252" t="s">
         <v>9</v>
@@ -18166,7 +18160,7 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B253" t="s">
         <v>9</v>
@@ -18180,7 +18174,7 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B254" t="s">
         <v>9</v>
@@ -18194,7 +18188,7 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B255" t="s">
         <v>9</v>
@@ -18208,7 +18202,7 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B256" t="s">
         <v>9</v>
@@ -18222,7 +18216,7 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B257" t="s">
         <v>9</v>
@@ -18236,7 +18230,7 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B258" t="s">
         <v>9</v>
@@ -18250,7 +18244,7 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B259" t="s">
         <v>9</v>
@@ -18264,7 +18258,7 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B260" t="s">
         <v>9</v>
@@ -18278,7 +18272,7 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B261" t="s">
         <v>9</v>
@@ -18292,7 +18286,7 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B262" t="s">
         <v>9</v>
@@ -18306,7 +18300,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B263" t="s">
         <v>9</v>
@@ -18320,7 +18314,7 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B264" t="s">
         <v>9</v>
@@ -18334,7 +18328,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B265" t="s">
         <v>9</v>
@@ -18348,7 +18342,7 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B266" t="s">
         <v>9</v>
@@ -18362,7 +18356,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B267" t="s">
         <v>9</v>
@@ -18376,7 +18370,7 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B268" t="s">
         <v>9</v>
@@ -18390,7 +18384,7 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B269" t="s">
         <v>9</v>
@@ -18404,7 +18398,7 @@
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B270" t="s">
         <v>9</v>
@@ -18418,7 +18412,7 @@
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B271" t="s">
         <v>9</v>
@@ -18438,7 +18432,7 @@
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18788,7 +18782,7 @@
         <v>9</v>
       </c>
       <c r="C297" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="D297" t="s">
         <v>35</v>
@@ -18858,7 +18852,7 @@
         <v>9</v>
       </c>
       <c r="C302" t="s">
-        <v>1353</v>
+        <v>1317</v>
       </c>
       <c r="D302" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
chore: sync project test execution reports, workflows, and configurations
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium-summary.xlsx
+++ b/selenium-tests/reports/selenium-summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1351">
   <si>
     <t>Metric</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:49 pm</t>
+    <t>6/8/2026, 9:42:10 am</t>
   </si>
   <si>
     <t>Target Browser</t>
@@ -49,7 +49,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>41.28 seconds</t>
+    <t>77.00 seconds</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -3949,127 +3949,124 @@
     <t>Execution Time (s)</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:11 pm</t>
-  </si>
-  <si>
-    <t>2.02s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:14 pm</t>
-  </si>
-  <si>
-    <t>2.83s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:17 pm</t>
-  </si>
-  <si>
-    <t>2.55s</t>
+    <t>6/8/2026, 9:41:06 am</t>
+  </si>
+  <si>
+    <t>2.37s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:09 am</t>
+  </si>
+  <si>
+    <t>2.81s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:11 am</t>
+  </si>
+  <si>
+    <t>2.79s</t>
   </si>
   <si>
     <t>0.15s</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:20 pm</t>
-  </si>
-  <si>
-    <t>2.75s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:21 pm</t>
-  </si>
-  <si>
-    <t>1.26s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:23 pm</t>
-  </si>
-  <si>
-    <t>2.35s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:26 pm</t>
-  </si>
-  <si>
-    <t>2.43s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:30 pm</t>
-  </si>
-  <si>
-    <t>4.52s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:32 pm</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:35 pm</t>
-  </si>
-  <si>
-    <t>2.87s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:38 pm</t>
-  </si>
-  <si>
-    <t>2.32s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:40 pm</t>
-  </si>
-  <si>
-    <t>2.63s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:43 pm</t>
-  </si>
-  <si>
-    <t>2.24s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:44 pm</t>
-  </si>
-  <si>
-    <t>0.53s</t>
-  </si>
-  <si>
-    <t>0.00s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:45 pm</t>
-  </si>
-  <si>
-    <t>0.78s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:46 pm</t>
-  </si>
-  <si>
-    <t>0.43s</t>
-  </si>
-  <si>
-    <t>28/7/2026, 9:39:47 pm</t>
-  </si>
-  <si>
-    <t>0.77s</t>
+    <t>6/8/2026, 9:41:14 am</t>
+  </si>
+  <si>
+    <t>0.20s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:17 am</t>
+  </si>
+  <si>
+    <t>2.36s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:25 am</t>
+  </si>
+  <si>
+    <t>8.04s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:27 am</t>
+  </si>
+  <si>
+    <t>2.34s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:30 am</t>
+  </si>
+  <si>
+    <t>2.28s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:37 am</t>
+  </si>
+  <si>
+    <t>7.20s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:40 am</t>
+  </si>
+  <si>
+    <t>3.62s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:47 am</t>
+  </si>
+  <si>
+    <t>6.21s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:41:52 am</t>
+  </si>
+  <si>
+    <t>2.26s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:01 am</t>
+  </si>
+  <si>
+    <t>0.57s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:02 am</t>
+  </si>
+  <si>
+    <t>0.40s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:03 am</t>
+  </si>
+  <si>
+    <t>0.42s</t>
   </si>
   <si>
     <t>0.41s</t>
   </si>
   <si>
-    <t>28/7/2026, 9:39:48 pm</t>
-  </si>
-  <si>
-    <t>0.30s</t>
-  </si>
-  <si>
-    <t>0.35s</t>
-  </si>
-  <si>
-    <t>0.33s</t>
-  </si>
-  <si>
-    <t>0.24s</t>
+    <t>6/8/2026, 9:42:04 am</t>
+  </si>
+  <si>
+    <t>0.45s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:05 am</t>
+  </si>
+  <si>
+    <t>0.39s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:06 am</t>
+  </si>
+  <si>
+    <t>0.44s</t>
+  </si>
+  <si>
+    <t>6/8/2026, 9:42:07 am</t>
+  </si>
+  <si>
+    <t>0.34s</t>
   </si>
 </sst>
 </file>
@@ -14722,7 +14719,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>1319</v>
+        <v>1314</v>
       </c>
       <c r="D7" t="s">
         <v>35</v>
@@ -14744,13 +14741,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="D9" t="s">
         <v>35</v>
@@ -14758,7 +14755,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -14772,13 +14769,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="D11" t="s">
         <v>35</v>
@@ -14786,13 +14783,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1324</v>
+        <v>1322</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
@@ -14800,13 +14797,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="D13" t="s">
         <v>35</v>
@@ -14814,7 +14811,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -14828,7 +14825,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -14842,7 +14839,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
@@ -14856,7 +14853,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
@@ -14870,7 +14867,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
@@ -14884,7 +14881,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -14898,7 +14895,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
@@ -14912,7 +14909,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -14926,7 +14923,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -14940,7 +14937,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
@@ -14954,7 +14951,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
@@ -14968,7 +14965,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
@@ -14982,7 +14979,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
@@ -14996,7 +14993,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
@@ -15010,7 +15007,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
@@ -15024,7 +15021,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
@@ -15038,7 +15035,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
@@ -15052,7 +15049,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
@@ -15066,13 +15063,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>1312</v>
+        <v>1327</v>
       </c>
       <c r="D32" t="s">
         <v>35</v>
@@ -15080,13 +15077,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
         <v>1329</v>
-      </c>
-      <c r="B33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1330</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -15094,7 +15091,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -15108,7 +15105,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
@@ -15122,7 +15119,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
@@ -15136,7 +15133,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -15150,7 +15147,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -15164,7 +15161,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -15178,7 +15175,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -15192,13 +15189,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
         <v>1331</v>
-      </c>
-      <c r="B41" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1332</v>
       </c>
       <c r="D41" t="s">
         <v>35</v>
@@ -15206,13 +15203,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>1332</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
         <v>1333</v>
-      </c>
-      <c r="B42" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" t="s">
-        <v>1334</v>
       </c>
       <c r="D42" t="s">
         <v>35</v>
@@ -15220,7 +15217,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -15234,7 +15231,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -15248,7 +15245,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -15262,7 +15259,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -15276,7 +15273,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -15290,7 +15287,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -15304,7 +15301,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -15318,7 +15315,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -15332,7 +15329,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -15346,7 +15343,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -15360,7 +15357,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -15374,7 +15371,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -15388,7 +15385,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -15402,7 +15399,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -15416,7 +15413,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B57" t="s">
         <v>9</v>
@@ -15430,7 +15427,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -15444,7 +15441,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
@@ -15458,7 +15455,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
@@ -15472,7 +15469,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B61" t="s">
         <v>9</v>
@@ -15486,13 +15483,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
         <v>1335</v>
-      </c>
-      <c r="B62" t="s">
-        <v>9</v>
-      </c>
-      <c r="C62" t="s">
-        <v>1336</v>
       </c>
       <c r="D62" t="s">
         <v>35</v>
@@ -15500,7 +15497,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -15514,7 +15511,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
@@ -15528,7 +15525,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -15542,7 +15539,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B66" t="s">
         <v>9</v>
@@ -15556,7 +15553,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -15570,7 +15567,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -15584,7 +15581,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -15598,7 +15595,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
@@ -15612,7 +15609,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B71" t="s">
         <v>9</v>
@@ -15626,7 +15623,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B72" t="s">
         <v>9</v>
@@ -15640,7 +15637,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
@@ -15654,7 +15651,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B74" t="s">
         <v>9</v>
@@ -15668,7 +15665,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B75" t="s">
         <v>9</v>
@@ -15682,7 +15679,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -15696,7 +15693,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
@@ -15710,7 +15707,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
@@ -15724,7 +15721,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
@@ -15738,7 +15735,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -15752,7 +15749,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
@@ -15766,13 +15763,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
         <v>1337</v>
-      </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
-      <c r="C82" t="s">
-        <v>1338</v>
       </c>
       <c r="D82" t="s">
         <v>35</v>
@@ -15780,13 +15777,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
       </c>
       <c r="C83" t="s">
-        <v>1339</v>
+        <v>1317</v>
       </c>
       <c r="D83" t="s">
         <v>35</v>
@@ -15794,7 +15791,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -15808,7 +15805,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -15822,7 +15819,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -15836,7 +15833,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B87" t="s">
         <v>9</v>
@@ -15850,7 +15847,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B88" t="s">
         <v>9</v>
@@ -15864,7 +15861,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -15878,7 +15875,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -15892,7 +15889,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -15906,7 +15903,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -15920,7 +15917,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B93" t="s">
         <v>9</v>
@@ -15934,7 +15931,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B94" t="s">
         <v>9</v>
@@ -15948,7 +15945,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B95" t="s">
         <v>9</v>
@@ -15962,7 +15959,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B96" t="s">
         <v>9</v>
@@ -15976,7 +15973,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -15990,7 +15987,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B98" t="s">
         <v>9</v>
@@ -16004,7 +16001,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -16018,7 +16015,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B100" t="s">
         <v>9</v>
@@ -16032,7 +16029,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -16046,7 +16043,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B102" t="s">
         <v>9</v>
@@ -16060,7 +16057,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B103" t="s">
         <v>9</v>
@@ -16074,7 +16071,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B104" t="s">
         <v>9</v>
@@ -16088,7 +16085,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -16102,7 +16099,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B106" t="s">
         <v>9</v>
@@ -16116,7 +16113,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
@@ -16130,7 +16127,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B108" t="s">
         <v>9</v>
@@ -16144,7 +16141,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B109" t="s">
         <v>9</v>
@@ -16158,7 +16155,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B110" t="s">
         <v>9</v>
@@ -16172,7 +16169,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -16186,13 +16183,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B112" t="s">
         <v>9</v>
       </c>
       <c r="C112" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="D112" t="s">
         <v>35</v>
@@ -16200,7 +16197,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B113" t="s">
         <v>9</v>
@@ -16214,7 +16211,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B114" t="s">
         <v>9</v>
@@ -16228,7 +16225,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B115" t="s">
         <v>9</v>
@@ -16242,7 +16239,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B116" t="s">
         <v>9</v>
@@ -16256,7 +16253,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B117" t="s">
         <v>9</v>
@@ -16270,7 +16267,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B118" t="s">
         <v>9</v>
@@ -16284,7 +16281,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B119" t="s">
         <v>9</v>
@@ -16298,7 +16295,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B120" t="s">
         <v>9</v>
@@ -16312,7 +16309,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B121" t="s">
         <v>9</v>
@@ -16326,7 +16323,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B122" t="s">
         <v>9</v>
@@ -16340,7 +16337,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B123" t="s">
         <v>9</v>
@@ -16354,7 +16351,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B124" t="s">
         <v>9</v>
@@ -16368,7 +16365,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B125" t="s">
         <v>9</v>
@@ -16382,7 +16379,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B126" t="s">
         <v>9</v>
@@ -16396,7 +16393,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B127" t="s">
         <v>9</v>
@@ -16410,7 +16407,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B128" t="s">
         <v>9</v>
@@ -16424,7 +16421,7 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B129" t="s">
         <v>9</v>
@@ -16438,7 +16435,7 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B130" t="s">
         <v>9</v>
@@ -16452,7 +16449,7 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B131" t="s">
         <v>9</v>
@@ -16466,7 +16463,7 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B132" t="s">
         <v>9</v>
@@ -16480,7 +16477,7 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B133" t="s">
         <v>9</v>
@@ -16494,7 +16491,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B134" t="s">
         <v>9</v>
@@ -16508,7 +16505,7 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B135" t="s">
         <v>9</v>
@@ -16522,7 +16519,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="B136" t="s">
         <v>9</v>
@@ -16536,13 +16533,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B137" t="s">
         <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="D137" t="s">
         <v>35</v>
@@ -16550,7 +16547,7 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B138" t="s">
         <v>9</v>
@@ -16564,7 +16561,7 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B139" t="s">
         <v>9</v>
@@ -16578,7 +16575,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B140" t="s">
         <v>9</v>
@@ -16592,7 +16589,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B141" t="s">
         <v>9</v>
@@ -16606,7 +16603,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B142" t="s">
         <v>9</v>
@@ -16620,7 +16617,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B143" t="s">
         <v>9</v>
@@ -16634,7 +16631,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B144" t="s">
         <v>9</v>
@@ -16648,7 +16645,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B145" t="s">
         <v>9</v>
@@ -16662,7 +16659,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B146" t="s">
         <v>9</v>
@@ -16676,7 +16673,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B147" t="s">
         <v>9</v>
@@ -16690,7 +16687,7 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B148" t="s">
         <v>9</v>
@@ -16704,7 +16701,7 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B149" t="s">
         <v>9</v>
@@ -16718,7 +16715,7 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B150" t="s">
         <v>9</v>
@@ -16732,7 +16729,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B151" t="s">
         <v>9</v>
@@ -16746,7 +16743,7 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
@@ -16760,7 +16757,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
@@ -16774,7 +16771,7 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
@@ -16788,7 +16785,7 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
@@ -16802,7 +16799,7 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
@@ -16816,7 +16813,7 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
@@ -16830,7 +16827,7 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
@@ -16844,7 +16841,7 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
@@ -16858,7 +16855,7 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
@@ -16872,7 +16869,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
@@ -16886,7 +16883,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
@@ -16900,7 +16897,7 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
@@ -16914,7 +16911,7 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
@@ -16928,7 +16925,7 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
@@ -16942,7 +16939,7 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
@@ -16956,13 +16953,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B167" t="s">
         <v>9</v>
       </c>
       <c r="C167" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="D167" t="s">
         <v>35</v>
@@ -16970,7 +16967,7 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
@@ -16984,7 +16981,7 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B169" t="s">
         <v>9</v>
@@ -16998,7 +16995,7 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B170" t="s">
         <v>9</v>
@@ -17012,7 +17009,7 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B171" t="s">
         <v>9</v>
@@ -17026,7 +17023,7 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B172" t="s">
         <v>9</v>
@@ -17040,7 +17037,7 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B173" t="s">
         <v>9</v>
@@ -17054,7 +17051,7 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B174" t="s">
         <v>9</v>
@@ -17068,7 +17065,7 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B175" t="s">
         <v>9</v>
@@ -17082,7 +17079,7 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B176" t="s">
         <v>9</v>
@@ -17096,7 +17093,7 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B177" t="s">
         <v>9</v>
@@ -17110,7 +17107,7 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B178" t="s">
         <v>9</v>
@@ -17124,7 +17121,7 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B179" t="s">
         <v>9</v>
@@ -17138,7 +17135,7 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B180" t="s">
         <v>9</v>
@@ -17152,7 +17149,7 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B181" t="s">
         <v>9</v>
@@ -17166,7 +17163,7 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B182" t="s">
         <v>9</v>
@@ -17180,7 +17177,7 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B183" t="s">
         <v>9</v>
@@ -17194,7 +17191,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B184" t="s">
         <v>9</v>
@@ -17208,7 +17205,7 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -17222,7 +17219,7 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -17236,7 +17233,7 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -17250,7 +17247,7 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B188" t="s">
         <v>9</v>
@@ -17264,7 +17261,7 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B189" t="s">
         <v>9</v>
@@ -17278,7 +17275,7 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B190" t="s">
         <v>9</v>
@@ -17292,7 +17289,7 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1344</v>
+        <v>1340</v>
       </c>
       <c r="B191" t="s">
         <v>9</v>
@@ -17306,13 +17303,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B192" t="s">
+        <v>9</v>
+      </c>
+      <c r="C192" t="s">
         <v>1344</v>
-      </c>
-      <c r="B192" t="s">
-        <v>9</v>
-      </c>
-      <c r="C192" t="s">
-        <v>1346</v>
       </c>
       <c r="D192" t="s">
         <v>35</v>
@@ -17320,7 +17317,7 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B193" t="s">
         <v>9</v>
@@ -17334,7 +17331,7 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B194" t="s">
         <v>9</v>
@@ -17348,7 +17345,7 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B195" t="s">
         <v>9</v>
@@ -17362,7 +17359,7 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B196" t="s">
         <v>9</v>
@@ -17376,7 +17373,7 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B197" t="s">
         <v>9</v>
@@ -17390,7 +17387,7 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B198" t="s">
         <v>9</v>
@@ -17404,7 +17401,7 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B199" t="s">
         <v>9</v>
@@ -17418,7 +17415,7 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B200" t="s">
         <v>9</v>
@@ -17432,7 +17429,7 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B201" t="s">
         <v>9</v>
@@ -17446,7 +17443,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B202" t="s">
         <v>9</v>
@@ -17460,7 +17457,7 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B203" t="s">
         <v>9</v>
@@ -17474,7 +17471,7 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B204" t="s">
         <v>9</v>
@@ -17488,7 +17485,7 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B205" t="s">
         <v>9</v>
@@ -17502,7 +17499,7 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B206" t="s">
         <v>9</v>
@@ -17516,7 +17513,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B207" t="s">
         <v>9</v>
@@ -17530,7 +17527,7 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B208" t="s">
         <v>9</v>
@@ -17544,7 +17541,7 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B209" t="s">
         <v>9</v>
@@ -17558,7 +17555,7 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B210" t="s">
         <v>9</v>
@@ -17572,7 +17569,7 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B211" t="s">
         <v>9</v>
@@ -17586,7 +17583,7 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B212" t="s">
         <v>9</v>
@@ -17600,7 +17597,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B213" t="s">
         <v>9</v>
@@ -17614,7 +17611,7 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B214" t="s">
         <v>9</v>
@@ -17628,7 +17625,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B215" t="s">
         <v>9</v>
@@ -17642,7 +17639,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B216" t="s">
         <v>9</v>
@@ -17656,7 +17653,7 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B217" t="s">
         <v>9</v>
@@ -17670,7 +17667,7 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B218" t="s">
         <v>9</v>
@@ -17684,7 +17681,7 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B219" t="s">
         <v>9</v>
@@ -17698,7 +17695,7 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B220" t="s">
         <v>9</v>
@@ -17712,7 +17709,7 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B221" t="s">
         <v>9</v>
@@ -17726,13 +17723,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B222" t="s">
         <v>9</v>
       </c>
       <c r="C222" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="D222" t="s">
         <v>35</v>
@@ -17740,7 +17737,7 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B223" t="s">
         <v>9</v>
@@ -17754,7 +17751,7 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B224" t="s">
         <v>9</v>
@@ -17768,7 +17765,7 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B225" t="s">
         <v>9</v>
@@ -17782,7 +17779,7 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B226" t="s">
         <v>9</v>
@@ -17796,7 +17793,7 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B227" t="s">
         <v>9</v>
@@ -17810,7 +17807,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B228" t="s">
         <v>9</v>
@@ -17824,7 +17821,7 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B229" t="s">
         <v>9</v>
@@ -17838,7 +17835,7 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B230" t="s">
         <v>9</v>
@@ -17852,7 +17849,7 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B231" t="s">
         <v>9</v>
@@ -17866,7 +17863,7 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B232" t="s">
         <v>9</v>
@@ -17880,7 +17877,7 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B233" t="s">
         <v>9</v>
@@ -17894,7 +17891,7 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B234" t="s">
         <v>9</v>
@@ -17908,7 +17905,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B235" t="s">
         <v>9</v>
@@ -17922,7 +17919,7 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B236" t="s">
         <v>9</v>
@@ -17936,7 +17933,7 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B237" t="s">
         <v>9</v>
@@ -17950,7 +17947,7 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B238" t="s">
         <v>9</v>
@@ -17964,7 +17961,7 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B239" t="s">
         <v>9</v>
@@ -17978,7 +17975,7 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B240" t="s">
         <v>9</v>
@@ -17992,7 +17989,7 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B241" t="s">
         <v>9</v>
@@ -18006,7 +18003,7 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B242" t="s">
         <v>9</v>
@@ -18020,7 +18017,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B243" t="s">
         <v>9</v>
@@ -18034,7 +18031,7 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B244" t="s">
         <v>9</v>
@@ -18048,7 +18045,7 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B245" t="s">
         <v>9</v>
@@ -18062,7 +18059,7 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B246" t="s">
         <v>9</v>
@@ -18082,7 +18079,7 @@
         <v>9</v>
       </c>
       <c r="C247" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="D247" t="s">
         <v>35</v>
@@ -18426,13 +18423,13 @@
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B272" t="s">
         <v>9</v>
       </c>
       <c r="C272" t="s">
-        <v>1350</v>
+        <v>1346</v>
       </c>
       <c r="D272" t="s">
         <v>35</v>
@@ -18440,7 +18437,7 @@
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B273" t="s">
         <v>9</v>
@@ -18454,7 +18451,7 @@
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B274" t="s">
         <v>9</v>
@@ -18468,7 +18465,7 @@
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B275" t="s">
         <v>9</v>
@@ -18482,7 +18479,7 @@
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B276" t="s">
         <v>9</v>
@@ -18496,7 +18493,7 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B277" t="s">
         <v>9</v>
@@ -18510,7 +18507,7 @@
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B278" t="s">
         <v>9</v>
@@ -18524,7 +18521,7 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B279" t="s">
         <v>9</v>
@@ -18538,7 +18535,7 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B280" t="s">
         <v>9</v>
@@ -18552,7 +18549,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B281" t="s">
         <v>9</v>
@@ -18566,7 +18563,7 @@
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B282" t="s">
         <v>9</v>
@@ -18580,7 +18577,7 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B283" t="s">
         <v>9</v>
@@ -18594,7 +18591,7 @@
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B284" t="s">
         <v>9</v>
@@ -18608,7 +18605,7 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B285" t="s">
         <v>9</v>
@@ -18622,7 +18619,7 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B286" t="s">
         <v>9</v>
@@ -18636,7 +18633,7 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B287" t="s">
         <v>9</v>
@@ -18650,7 +18647,7 @@
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B288" t="s">
         <v>9</v>
@@ -18664,7 +18661,7 @@
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B289" t="s">
         <v>9</v>
@@ -18678,7 +18675,7 @@
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B290" t="s">
         <v>9</v>
@@ -18692,7 +18689,7 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B291" t="s">
         <v>9</v>
@@ -18706,7 +18703,7 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B292" t="s">
         <v>9</v>
@@ -18720,7 +18717,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B293" t="s">
         <v>9</v>
@@ -18734,7 +18731,7 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B294" t="s">
         <v>9</v>
@@ -18748,7 +18745,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B295" t="s">
         <v>9</v>
@@ -18762,7 +18759,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>7</v>
+        <v>1349</v>
       </c>
       <c r="B296" t="s">
         <v>9</v>
@@ -18782,7 +18779,7 @@
         <v>9</v>
       </c>
       <c r="C297" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="D297" t="s">
         <v>35</v>

</xml_diff>